<commit_message>
Upgrade Pattern Mastery: Mastered/Total + Representative Problems
- "Problems Solved" → "Mastered / Total" (e.g. "— / 11" for Sliding
  Window, "— / 22" for DP) — shows progress as fraction, not just count
- New column "Representative Problems" pre-filled with best LC numbers
  per pattern (e.g. Sliding Window → LC 3, 76, 424, 438, 567, 239, 121)
- Makes revision faster: glance at representative problems to instantly
  recall the pattern's core techniques

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Interview-Preparation-Tracker.xlsx
+++ b/Interview-Preparation-Tracker.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,6 +126,11 @@
       <color rgb="00FBBF24"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="0022D3EE"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -160,7 +165,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -215,11 +220,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="002D3748"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="002D3748"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -306,6 +322,13 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6931,7 +6954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J352"/>
+  <dimension ref="A1:K352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6942,8 +6965,9 @@
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7012,6 +7036,7 @@
         <f>IF(COUNTA(H10:H35)&gt;0,ROUND(AVERAGE(H10:H35),1),"—")</f>
         <v/>
       </c>
+      <c r="K5" s="32" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
@@ -7045,6 +7070,7 @@
       </c>
       <c r="I6" s="28" t="n"/>
       <c r="J6" s="28" t="n"/>
+      <c r="K6" s="28" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
@@ -7061,7 +7087,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Problems Solved</t>
+          <t>Mastered / Total</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -7102,6 +7128,11 @@
       <c r="J9" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Representative Problems</t>
         </is>
       </c>
     </row>
@@ -7111,7 +7142,11 @@
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>— / 7</t>
+        </is>
+      </c>
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n"/>
@@ -7120,6 +7155,11 @@
       <c r="H10" s="5" t="n"/>
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
+      <c r="K10" s="33" t="inlineStr">
+        <is>
+          <t>LC 1, 49, 238, 128, 347, 48, 54</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -7127,7 +7167,11 @@
           <t>Prefix Sum</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
       <c r="E11" s="7" t="n"/>
@@ -7136,6 +7180,11 @@
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
+      <c r="K11" s="34" t="inlineStr">
+        <is>
+          <t>LC 303, 560, 974, 1314</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -7143,7 +7192,11 @@
           <t>Two Pointers</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>— / 5</t>
+        </is>
+      </c>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="5" t="n"/>
       <c r="E12" s="5" t="n"/>
@@ -7152,6 +7205,11 @@
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
+      <c r="K12" s="33" t="inlineStr">
+        <is>
+          <t>LC 11, 15, 75, 287, 5</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -7159,7 +7217,11 @@
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>— / 11</t>
+        </is>
+      </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
@@ -7168,6 +7230,11 @@
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
+      <c r="K13" s="34" t="inlineStr">
+        <is>
+          <t>LC 3, 76, 424, 438, 567, 239, 121</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -7175,7 +7242,11 @@
           <t>Binary Search</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>— / 10</t>
+        </is>
+      </c>
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="5" t="n"/>
       <c r="E14" s="5" t="n"/>
@@ -7184,6 +7255,11 @@
       <c r="H14" s="5" t="n"/>
       <c r="I14" s="5" t="n"/>
       <c r="J14" s="5" t="n"/>
+      <c r="K14" s="33" t="inlineStr">
+        <is>
+          <t>LC 33, 875, 410, 4, 34, 153, 378</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -7191,7 +7267,11 @@
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>— / 4</t>
+        </is>
+      </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
       <c r="E15" s="7" t="n"/>
@@ -7200,6 +7280,11 @@
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="n"/>
+      <c r="K15" s="34" t="inlineStr">
+        <is>
+          <t>LC 136, 191, 338, 371</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -7207,7 +7292,11 @@
           <t>Stack</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>— / 8</t>
+        </is>
+      </c>
       <c r="C16" s="5" t="n"/>
       <c r="D16" s="5" t="n"/>
       <c r="E16" s="5" t="n"/>
@@ -7216,6 +7305,11 @@
       <c r="H16" s="5" t="n"/>
       <c r="I16" s="5" t="n"/>
       <c r="J16" s="5" t="n"/>
+      <c r="K16" s="33" t="inlineStr">
+        <is>
+          <t>LC 739, 84, 42, 394, 402, 907</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -7223,7 +7317,11 @@
           <t>Monotonic Stack</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
       <c r="E17" s="7" t="n"/>
@@ -7232,6 +7330,11 @@
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
+      <c r="K17" s="34" t="inlineStr">
+        <is>
+          <t>LC 739, 84, 503, 907, 901</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -7239,7 +7342,11 @@
           <t>Queue</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C18" s="5" t="n"/>
       <c r="D18" s="5" t="n"/>
       <c r="E18" s="5" t="n"/>
@@ -7248,6 +7355,11 @@
       <c r="H18" s="5" t="n"/>
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
+      <c r="K18" s="33" t="inlineStr">
+        <is>
+          <t>LC 239, 622, 346</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -7255,7 +7367,11 @@
           <t>Heap / Priority Queue</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>— / 7</t>
+        </is>
+      </c>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
       <c r="E19" s="7" t="n"/>
@@ -7264,6 +7380,11 @@
       <c r="H19" s="7" t="n"/>
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
+      <c r="K19" s="34" t="inlineStr">
+        <is>
+          <t>LC 215, 295, 253, 23, 632, 973</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -7271,7 +7392,11 @@
           <t>Linked List</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>— / 7</t>
+        </is>
+      </c>
       <c r="C20" s="5" t="n"/>
       <c r="D20" s="5" t="n"/>
       <c r="E20" s="5" t="n"/>
@@ -7280,6 +7405,11 @@
       <c r="H20" s="5" t="n"/>
       <c r="I20" s="5" t="n"/>
       <c r="J20" s="5" t="n"/>
+      <c r="K20" s="33" t="inlineStr">
+        <is>
+          <t>LC 206, 141, 19, 2, 25, 143, 138</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -7287,7 +7417,11 @@
           <t>Fast &amp; Slow Pointer</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
@@ -7296,6 +7430,11 @@
       <c r="H21" s="7" t="n"/>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
+      <c r="K21" s="34" t="inlineStr">
+        <is>
+          <t>LC 141, 142, 287, 876, 202</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -7303,7 +7442,11 @@
           <t>Trees (DFS)</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>— / 15</t>
+        </is>
+      </c>
       <c r="C22" s="5" t="n"/>
       <c r="D22" s="5" t="n"/>
       <c r="E22" s="5" t="n"/>
@@ -7312,6 +7455,11 @@
       <c r="H22" s="5" t="n"/>
       <c r="I22" s="5" t="n"/>
       <c r="J22" s="5" t="n"/>
+      <c r="K22" s="33" t="inlineStr">
+        <is>
+          <t>LC 124, 543, 297, 236, 105, 114</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -7319,7 +7467,11 @@
           <t>Trees (BFS)</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
       <c r="E23" s="7" t="n"/>
@@ -7328,6 +7480,11 @@
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
+      <c r="K23" s="34" t="inlineStr">
+        <is>
+          <t>LC 102, 199, 863, 637</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -7335,7 +7492,11 @@
           <t>Binary Search Tree</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C24" s="5" t="n"/>
       <c r="D24" s="5" t="n"/>
       <c r="E24" s="5" t="n"/>
@@ -7344,6 +7505,11 @@
       <c r="H24" s="5" t="n"/>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
+      <c r="K24" s="33" t="inlineStr">
+        <is>
+          <t>LC 98, 230, 235, 701</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -7351,7 +7517,11 @@
           <t>Graph DFS</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>— / 20</t>
+        </is>
+      </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
       <c r="E25" s="7" t="n"/>
@@ -7360,6 +7530,11 @@
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
+      <c r="K25" s="34" t="inlineStr">
+        <is>
+          <t>LC 200, 695, 417, 207, 133, 802</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -7367,7 +7542,11 @@
           <t>Graph BFS</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n"/>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C26" s="5" t="n"/>
       <c r="D26" s="5" t="n"/>
       <c r="E26" s="5" t="n"/>
@@ -7376,6 +7555,11 @@
       <c r="H26" s="5" t="n"/>
       <c r="I26" s="5" t="n"/>
       <c r="J26" s="5" t="n"/>
+      <c r="K26" s="33" t="inlineStr">
+        <is>
+          <t>LC 994, 127, 286, 1091</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -7383,7 +7567,11 @@
           <t>Topological Sort</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="7" t="n"/>
       <c r="E27" s="7" t="n"/>
@@ -7392,6 +7580,11 @@
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
+      <c r="K27" s="34" t="inlineStr">
+        <is>
+          <t>LC 207, 210, 269, 2115</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -7399,7 +7592,11 @@
           <t>Union Find (Disjoint Set)</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C28" s="5" t="n"/>
       <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="n"/>
@@ -7408,6 +7605,11 @@
       <c r="H28" s="5" t="n"/>
       <c r="I28" s="5" t="n"/>
       <c r="J28" s="5" t="n"/>
+      <c r="K28" s="33" t="inlineStr">
+        <is>
+          <t>LC 547, 684, 721, 323, 1584</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -7415,7 +7617,11 @@
           <t>Trie</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="7" t="n"/>
       <c r="E29" s="7" t="n"/>
@@ -7424,6 +7630,11 @@
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="7" t="n"/>
+      <c r="K29" s="34" t="inlineStr">
+        <is>
+          <t>LC 208, 211, 212, 642</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -7431,7 +7642,11 @@
           <t>Backtracking</t>
         </is>
       </c>
-      <c r="B30" s="5" t="n"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>— / 6</t>
+        </is>
+      </c>
       <c r="C30" s="5" t="n"/>
       <c r="D30" s="5" t="n"/>
       <c r="E30" s="5" t="n"/>
@@ -7440,6 +7655,11 @@
       <c r="H30" s="5" t="n"/>
       <c r="I30" s="5" t="n"/>
       <c r="J30" s="5" t="n"/>
+      <c r="K30" s="33" t="inlineStr">
+        <is>
+          <t>LC 39, 46, 78, 79, 22, 51</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -7447,7 +7667,11 @@
           <t>Greedy</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>— / 5</t>
+        </is>
+      </c>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="7" t="n"/>
       <c r="E31" s="7" t="n"/>
@@ -7456,6 +7680,11 @@
       <c r="H31" s="7" t="n"/>
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="7" t="n"/>
+      <c r="K31" s="34" t="inlineStr">
+        <is>
+          <t>LC 55, 45, 53, 621, 134</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -7463,7 +7692,11 @@
           <t>Dynamic Programming</t>
         </is>
       </c>
-      <c r="B32" s="5" t="n"/>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>— / 22</t>
+        </is>
+      </c>
       <c r="C32" s="5" t="n"/>
       <c r="D32" s="5" t="n"/>
       <c r="E32" s="5" t="n"/>
@@ -7472,6 +7705,11 @@
       <c r="H32" s="5" t="n"/>
       <c r="I32" s="5" t="n"/>
       <c r="J32" s="5" t="n"/>
+      <c r="K32" s="33" t="inlineStr">
+        <is>
+          <t>LC 322, 72, 300, 1143, 198, 312, 152, 329</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -7479,7 +7717,11 @@
           <t>Interval Problems</t>
         </is>
       </c>
-      <c r="B33" s="7" t="n"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>— / 4</t>
+        </is>
+      </c>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="7" t="n"/>
       <c r="E33" s="7" t="n"/>
@@ -7488,6 +7730,11 @@
       <c r="H33" s="7" t="n"/>
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
+      <c r="K33" s="34" t="inlineStr">
+        <is>
+          <t>LC 56, 57, 435, 252, 253</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -7495,7 +7742,11 @@
           <t>Matrix Problems</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="C34" s="5" t="n"/>
       <c r="D34" s="5" t="n"/>
       <c r="E34" s="5" t="n"/>
@@ -7504,6 +7755,11 @@
       <c r="H34" s="5" t="n"/>
       <c r="I34" s="5" t="n"/>
       <c r="J34" s="5" t="n"/>
+      <c r="K34" s="33" t="inlineStr">
+        <is>
+          <t>LC 48, 54, 73, 74</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -7511,7 +7767,11 @@
           <t>Design Problems</t>
         </is>
       </c>
-      <c r="B35" s="7" t="n"/>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>— / 11</t>
+        </is>
+      </c>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="7" t="n"/>
       <c r="E35" s="7" t="n"/>
@@ -7520,6 +7780,11 @@
       <c r="H35" s="7" t="n"/>
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
+      <c r="K35" s="34" t="inlineStr">
+        <is>
+          <t>LC 146, 460, 208, 380, 981, 706, 642, 212</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
@@ -11694,39 +11959,39 @@
   <mergeCells count="36">
     <mergeCell ref="A312:D312"/>
     <mergeCell ref="A263:D263"/>
-    <mergeCell ref="A8:J8"/>
     <mergeCell ref="A159:D159"/>
     <mergeCell ref="A234:D234"/>
     <mergeCell ref="A206:D206"/>
     <mergeCell ref="A96:D96"/>
     <mergeCell ref="A324:D324"/>
-    <mergeCell ref="A4:J4"/>
     <mergeCell ref="A117:D117"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="A127:D127"/>
     <mergeCell ref="A186:D186"/>
+    <mergeCell ref="A66:K66"/>
     <mergeCell ref="A107:D107"/>
     <mergeCell ref="A178:D178"/>
     <mergeCell ref="A291:D291"/>
+    <mergeCell ref="A37:K37"/>
     <mergeCell ref="A138:D138"/>
     <mergeCell ref="A225:D225"/>
     <mergeCell ref="A334:D334"/>
-    <mergeCell ref="A1:J1"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="A343:D343"/>
     <mergeCell ref="A168:D168"/>
+    <mergeCell ref="A95:K95"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A196:D196"/>
     <mergeCell ref="A243:D243"/>
-    <mergeCell ref="A66:J66"/>
+    <mergeCell ref="A8:K8"/>
     <mergeCell ref="A282:D282"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A37:J37"/>
+    <mergeCell ref="A4:K4"/>
     <mergeCell ref="A149:D149"/>
     <mergeCell ref="A214:D214"/>
     <mergeCell ref="A272:D272"/>
     <mergeCell ref="A302:D302"/>
-    <mergeCell ref="A95:J95"/>
-    <mergeCell ref="A2:J2"/>
     <mergeCell ref="A254:D254"/>
   </mergeCells>
   <conditionalFormatting sqref="C10:C35">

</xml_diff>

<commit_message>
Switch to phased time allocation: DSA-heavy first, balanced later
Phase 1 (Months 1-4): DSA 45%, SD 25%, Java 15%, Kafka 10%, Cloud 5%
Phase 2 (Months 5-8): SD 30%, Java 25%, DSA 20%, Kafka 15%, Cloud 10%

Rationale: DSA is the gating round at Tier-1 companies — front-loading
it maximizes interview readiness. Once patterns are solid, shift weight
toward system design and backend depth for senior-level rounds.

Updated in both Dashboard sheet and BACKEND-ENGINEER-ROADMAP.md.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Interview-Preparation-Tracker.xlsx
+++ b/Interview-Preparation-Tracker.xlsx
@@ -165,7 +165,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -212,17 +212,6 @@
       <right style="thin">
         <color rgb="002D3748"/>
       </right>
-      <top style="thin">
-        <color rgb="002D3748"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="002D3748"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="002D3748"/>
       </top>
@@ -311,6 +300,7 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -318,17 +308,16 @@
     <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -736,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -769,7 +758,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TRACK ALLOCATION</t>
+          <t>PHASE 1: DSA-HEAVY (Months 1–4) — DSA is the gating round at Tier-1 companies</t>
         </is>
       </c>
     </row>
@@ -791,7 +780,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Focus</t>
         </is>
       </c>
     </row>
@@ -803,24 +792,24 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>~4.5h</t>
+          <t>~6.75h</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>142 problems</t>
+          <t>142 problems — highest interview impact</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Java &amp; Backend</t>
+          <t>System Design + DDIA</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -835,29 +824,29 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>3 sub-tracks</t>
+          <t>DDIA Ch 1-6 + 3 HLD designs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>System Design + DDIA</t>
+          <t>Java &amp; Backend</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>~3.75h</t>
+          <t>~2.25h</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>9 chapters + 8 designs</t>
+          <t>Effective Java + Design Patterns started</t>
         </is>
       </c>
     </row>
@@ -879,7 +868,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>11 + 5 topics</t>
+          <t>Kafka fundamentals + consumers</t>
         </is>
       </c>
     </row>
@@ -891,310 +880,449 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>~1.5h</t>
+          <t>~0.75h</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>5 technologies</t>
+          <t>Docker basics</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>MONTHLY MILESTONES</t>
+          <t>PHASE 2: BALANCED (Months 5–8) — After DSA patterns are solid</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Hrs/Wk</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Focus</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>DSA</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>~3h</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Revision + hard problems + mock interviews</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>System Design + DDIA</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>~4.5h</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>DDIA Ch 7-9 + 5 HLD designs + mocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Java &amp; Backend</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>~3.75h</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Design Patterns done + Spring Boot deep dive</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Kafka &amp; Redis</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>~2.25h</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Kafka reliability + Redis patterns</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Cloud &amp; Platform</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>~1.5h</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>K8s, OpenShift, CI/CD, AWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>MONTHLY MILESTONES</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>DSA</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Java &amp; Backend</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>System Design</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Kafka/Redis</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Cloud/Platform</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Month 1</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Phase 1: Arrays, Two Pointers, SW</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Effective Java started</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>DDIA Ch 1-2</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Kafka fundamentals</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Docker basics</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Month 2</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Phase 1-2: BS, Stack, Heap</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Effective Java 50%</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>DDIA Ch 3-4</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Kafka consumers</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Docker multi-stage</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
         <is>
           <t>Month 3</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Phase 2: LL, Intervals</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Effective Java done</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>DDIA Ch 5 + URL Shortener</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
         <is>
           <t>Kafka reliability</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>K8s basics</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Month 4</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Phase 3: Trees</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Design Patterns started</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>DDIA Ch 6 + Rate Limiter</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>Redis fundamentals</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>K8s probes/HPA</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>Month 5</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Phase 3: Graphs</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Design Patterns 50%</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>DDIA Ch 7 + Notification Sys</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Redis locking</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>OpenShift basics</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Month 6</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Phase 4: DP</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Design Patterns done</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>DDIA Ch 8-9 + Inventory</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>Integration practice</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>CI/CD pipelines</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>Month 7</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Phase 4-5: Greedy, BT, Design</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Spring Boot deep dive</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>Payment Sys + Search</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>E2E design</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>AWS fundamentals</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Month 8</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Review + Mocks</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Spring Security</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Dist Cache + Review</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Mock interviews</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Mock interviews</t>
         </is>
@@ -7036,10 +7164,10 @@
         <f>IF(COUNTA(H10:H35)&gt;0,ROUND(AVERAGE(H10:H35),1),"—")</f>
         <v/>
       </c>
-      <c r="K5" s="32" t="n"/>
+      <c r="K5" s="27" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Strongest Pattern</t>
         </is>
@@ -7048,8 +7176,8 @@
         <f>IF(COUNTA(H10:H35)&gt;0,INDEX(A10:A35,MATCH(MAX(H10:H35),H10:H35,0)),"—")</f>
         <v/>
       </c>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="27" t="inlineStr">
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>Weakest Pattern</t>
         </is>
@@ -7058,19 +7186,19 @@
         <f>IF(COUNTA(H10:H35)&gt;0,INDEX(A10:A35,MATCH(MIN(H10:H35),H10:H35,0)),"—")</f>
         <v/>
       </c>
-      <c r="F6" s="28" t="n"/>
-      <c r="G6" s="27" t="inlineStr">
+      <c r="F6" s="29" t="n"/>
+      <c r="G6" s="28" t="inlineStr">
         <is>
           <t>Completion %</t>
         </is>
       </c>
-      <c r="H6" s="29">
+      <c r="H6" s="30">
         <f>IF(COUNTA(H10:H35)&gt;0,ROUND(COUNTIF(H10:H35,"&gt;=4")/26*100,0)&amp;"%","0%")</f>
         <v/>
       </c>
-      <c r="I6" s="28" t="n"/>
-      <c r="J6" s="28" t="n"/>
-      <c r="K6" s="28" t="n"/>
+      <c r="I6" s="29" t="n"/>
+      <c r="J6" s="29" t="n"/>
+      <c r="K6" s="29" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="23" t="inlineStr">
@@ -7155,7 +7283,7 @@
       <c r="H10" s="5" t="n"/>
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
-      <c r="K10" s="33" t="inlineStr">
+      <c r="K10" s="31" t="inlineStr">
         <is>
           <t>LC 1, 49, 238, 128, 347, 48, 54</t>
         </is>
@@ -7180,7 +7308,7 @@
       <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
-      <c r="K11" s="34" t="inlineStr">
+      <c r="K11" s="32" t="inlineStr">
         <is>
           <t>LC 303, 560, 974, 1314</t>
         </is>
@@ -7205,7 +7333,7 @@
       <c r="H12" s="5" t="n"/>
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
-      <c r="K12" s="33" t="inlineStr">
+      <c r="K12" s="31" t="inlineStr">
         <is>
           <t>LC 11, 15, 75, 287, 5</t>
         </is>
@@ -7230,7 +7358,7 @@
       <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
-      <c r="K13" s="34" t="inlineStr">
+      <c r="K13" s="32" t="inlineStr">
         <is>
           <t>LC 3, 76, 424, 438, 567, 239, 121</t>
         </is>
@@ -7255,7 +7383,7 @@
       <c r="H14" s="5" t="n"/>
       <c r="I14" s="5" t="n"/>
       <c r="J14" s="5" t="n"/>
-      <c r="K14" s="33" t="inlineStr">
+      <c r="K14" s="31" t="inlineStr">
         <is>
           <t>LC 33, 875, 410, 4, 34, 153, 378</t>
         </is>
@@ -7280,7 +7408,7 @@
       <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="n"/>
-      <c r="K15" s="34" t="inlineStr">
+      <c r="K15" s="32" t="inlineStr">
         <is>
           <t>LC 136, 191, 338, 371</t>
         </is>
@@ -7305,7 +7433,7 @@
       <c r="H16" s="5" t="n"/>
       <c r="I16" s="5" t="n"/>
       <c r="J16" s="5" t="n"/>
-      <c r="K16" s="33" t="inlineStr">
+      <c r="K16" s="31" t="inlineStr">
         <is>
           <t>LC 739, 84, 42, 394, 402, 907</t>
         </is>
@@ -7330,7 +7458,7 @@
       <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
-      <c r="K17" s="34" t="inlineStr">
+      <c r="K17" s="32" t="inlineStr">
         <is>
           <t>LC 739, 84, 503, 907, 901</t>
         </is>
@@ -7355,7 +7483,7 @@
       <c r="H18" s="5" t="n"/>
       <c r="I18" s="5" t="n"/>
       <c r="J18" s="5" t="n"/>
-      <c r="K18" s="33" t="inlineStr">
+      <c r="K18" s="31" t="inlineStr">
         <is>
           <t>LC 239, 622, 346</t>
         </is>
@@ -7380,7 +7508,7 @@
       <c r="H19" s="7" t="n"/>
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
-      <c r="K19" s="34" t="inlineStr">
+      <c r="K19" s="32" t="inlineStr">
         <is>
           <t>LC 215, 295, 253, 23, 632, 973</t>
         </is>
@@ -7405,7 +7533,7 @@
       <c r="H20" s="5" t="n"/>
       <c r="I20" s="5" t="n"/>
       <c r="J20" s="5" t="n"/>
-      <c r="K20" s="33" t="inlineStr">
+      <c r="K20" s="31" t="inlineStr">
         <is>
           <t>LC 206, 141, 19, 2, 25, 143, 138</t>
         </is>
@@ -7430,7 +7558,7 @@
       <c r="H21" s="7" t="n"/>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="34" t="inlineStr">
+      <c r="K21" s="32" t="inlineStr">
         <is>
           <t>LC 141, 142, 287, 876, 202</t>
         </is>
@@ -7455,7 +7583,7 @@
       <c r="H22" s="5" t="n"/>
       <c r="I22" s="5" t="n"/>
       <c r="J22" s="5" t="n"/>
-      <c r="K22" s="33" t="inlineStr">
+      <c r="K22" s="31" t="inlineStr">
         <is>
           <t>LC 124, 543, 297, 236, 105, 114</t>
         </is>
@@ -7480,7 +7608,7 @@
       <c r="H23" s="7" t="n"/>
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
-      <c r="K23" s="34" t="inlineStr">
+      <c r="K23" s="32" t="inlineStr">
         <is>
           <t>LC 102, 199, 863, 637</t>
         </is>
@@ -7505,7 +7633,7 @@
       <c r="H24" s="5" t="n"/>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
-      <c r="K24" s="33" t="inlineStr">
+      <c r="K24" s="31" t="inlineStr">
         <is>
           <t>LC 98, 230, 235, 701</t>
         </is>
@@ -7530,7 +7658,7 @@
       <c r="H25" s="7" t="n"/>
       <c r="I25" s="7" t="n"/>
       <c r="J25" s="7" t="n"/>
-      <c r="K25" s="34" t="inlineStr">
+      <c r="K25" s="32" t="inlineStr">
         <is>
           <t>LC 200, 695, 417, 207, 133, 802</t>
         </is>
@@ -7555,7 +7683,7 @@
       <c r="H26" s="5" t="n"/>
       <c r="I26" s="5" t="n"/>
       <c r="J26" s="5" t="n"/>
-      <c r="K26" s="33" t="inlineStr">
+      <c r="K26" s="31" t="inlineStr">
         <is>
           <t>LC 994, 127, 286, 1091</t>
         </is>
@@ -7580,7 +7708,7 @@
       <c r="H27" s="7" t="n"/>
       <c r="I27" s="7" t="n"/>
       <c r="J27" s="7" t="n"/>
-      <c r="K27" s="34" t="inlineStr">
+      <c r="K27" s="32" t="inlineStr">
         <is>
           <t>LC 207, 210, 269, 2115</t>
         </is>
@@ -7605,7 +7733,7 @@
       <c r="H28" s="5" t="n"/>
       <c r="I28" s="5" t="n"/>
       <c r="J28" s="5" t="n"/>
-      <c r="K28" s="33" t="inlineStr">
+      <c r="K28" s="31" t="inlineStr">
         <is>
           <t>LC 547, 684, 721, 323, 1584</t>
         </is>
@@ -7630,7 +7758,7 @@
       <c r="H29" s="7" t="n"/>
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="7" t="n"/>
-      <c r="K29" s="34" t="inlineStr">
+      <c r="K29" s="32" t="inlineStr">
         <is>
           <t>LC 208, 211, 212, 642</t>
         </is>
@@ -7655,7 +7783,7 @@
       <c r="H30" s="5" t="n"/>
       <c r="I30" s="5" t="n"/>
       <c r="J30" s="5" t="n"/>
-      <c r="K30" s="33" t="inlineStr">
+      <c r="K30" s="31" t="inlineStr">
         <is>
           <t>LC 39, 46, 78, 79, 22, 51</t>
         </is>
@@ -7680,7 +7808,7 @@
       <c r="H31" s="7" t="n"/>
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="7" t="n"/>
-      <c r="K31" s="34" t="inlineStr">
+      <c r="K31" s="32" t="inlineStr">
         <is>
           <t>LC 55, 45, 53, 621, 134</t>
         </is>
@@ -7705,7 +7833,7 @@
       <c r="H32" s="5" t="n"/>
       <c r="I32" s="5" t="n"/>
       <c r="J32" s="5" t="n"/>
-      <c r="K32" s="33" t="inlineStr">
+      <c r="K32" s="31" t="inlineStr">
         <is>
           <t>LC 322, 72, 300, 1143, 198, 312, 152, 329</t>
         </is>
@@ -7730,7 +7858,7 @@
       <c r="H33" s="7" t="n"/>
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
-      <c r="K33" s="34" t="inlineStr">
+      <c r="K33" s="32" t="inlineStr">
         <is>
           <t>LC 56, 57, 435, 252, 253</t>
         </is>
@@ -7755,7 +7883,7 @@
       <c r="H34" s="5" t="n"/>
       <c r="I34" s="5" t="n"/>
       <c r="J34" s="5" t="n"/>
-      <c r="K34" s="33" t="inlineStr">
+      <c r="K34" s="31" t="inlineStr">
         <is>
           <t>LC 48, 54, 73, 74</t>
         </is>
@@ -7780,7 +7908,7 @@
       <c r="H35" s="7" t="n"/>
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
-      <c r="K35" s="34" t="inlineStr">
+      <c r="K35" s="32" t="inlineStr">
         <is>
           <t>LC 146, 460, 208, 380, 981, 706, 642, 212</t>
         </is>
@@ -8964,14 +9092,14 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="30" t="inlineStr">
+      <c r="A96" s="33" t="inlineStr">
         <is>
           <t>Arrays &amp; Hashing</t>
         </is>
       </c>
-      <c r="B96" s="31" t="n"/>
-      <c r="C96" s="31" t="n"/>
-      <c r="D96" s="31" t="n"/>
+      <c r="B96" s="34" t="n"/>
+      <c r="C96" s="34" t="n"/>
+      <c r="D96" s="34" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -9092,14 +9220,14 @@
       <c r="D105" s="7" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="30" t="inlineStr">
+      <c r="A107" s="33" t="inlineStr">
         <is>
           <t>Prefix Sum</t>
         </is>
       </c>
-      <c r="B107" s="31" t="n"/>
-      <c r="C107" s="31" t="n"/>
-      <c r="D107" s="31" t="n"/>
+      <c r="B107" s="34" t="n"/>
+      <c r="C107" s="34" t="n"/>
+      <c r="D107" s="34" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -9208,14 +9336,14 @@
       <c r="D115" s="5" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="30" t="inlineStr">
+      <c r="A117" s="33" t="inlineStr">
         <is>
           <t>Two Pointers</t>
         </is>
       </c>
-      <c r="B117" s="31" t="n"/>
-      <c r="C117" s="31" t="n"/>
-      <c r="D117" s="31" t="n"/>
+      <c r="B117" s="34" t="n"/>
+      <c r="C117" s="34" t="n"/>
+      <c r="D117" s="34" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
@@ -9324,14 +9452,14 @@
       <c r="D125" s="5" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="30" t="inlineStr">
+      <c r="A127" s="33" t="inlineStr">
         <is>
           <t>Sliding Window</t>
         </is>
       </c>
-      <c r="B127" s="31" t="n"/>
-      <c r="C127" s="31" t="n"/>
-      <c r="D127" s="31" t="n"/>
+      <c r="B127" s="34" t="n"/>
+      <c r="C127" s="34" t="n"/>
+      <c r="D127" s="34" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="inlineStr">
@@ -9452,14 +9580,14 @@
       <c r="D136" s="7" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="30" t="inlineStr">
+      <c r="A138" s="33" t="inlineStr">
         <is>
           <t>Binary Search</t>
         </is>
       </c>
-      <c r="B138" s="31" t="n"/>
-      <c r="C138" s="31" t="n"/>
-      <c r="D138" s="31" t="n"/>
+      <c r="B138" s="34" t="n"/>
+      <c r="C138" s="34" t="n"/>
+      <c r="D138" s="34" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="inlineStr">
@@ -9580,14 +9708,14 @@
       <c r="D147" s="7" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="30" t="inlineStr">
+      <c r="A149" s="33" t="inlineStr">
         <is>
           <t>Bit Manipulation</t>
         </is>
       </c>
-      <c r="B149" s="31" t="n"/>
-      <c r="C149" s="31" t="n"/>
-      <c r="D149" s="31" t="n"/>
+      <c r="B149" s="34" t="n"/>
+      <c r="C149" s="34" t="n"/>
+      <c r="D149" s="34" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -9696,14 +9824,14 @@
       <c r="D157" s="5" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="30" t="inlineStr">
+      <c r="A159" s="33" t="inlineStr">
         <is>
           <t>Stack</t>
         </is>
       </c>
-      <c r="B159" s="31" t="n"/>
-      <c r="C159" s="31" t="n"/>
-      <c r="D159" s="31" t="n"/>
+      <c r="B159" s="34" t="n"/>
+      <c r="C159" s="34" t="n"/>
+      <c r="D159" s="34" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -9800,14 +9928,14 @@
       <c r="D166" s="7" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="30" t="inlineStr">
+      <c r="A168" s="33" t="inlineStr">
         <is>
           <t>Monotonic Stack</t>
         </is>
       </c>
-      <c r="B168" s="31" t="n"/>
-      <c r="C168" s="31" t="n"/>
-      <c r="D168" s="31" t="n"/>
+      <c r="B168" s="34" t="n"/>
+      <c r="C168" s="34" t="n"/>
+      <c r="D168" s="34" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="inlineStr">
@@ -9916,14 +10044,14 @@
       <c r="D176" s="5" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="30" t="inlineStr">
+      <c r="A178" s="33" t="inlineStr">
         <is>
           <t>Queue</t>
         </is>
       </c>
-      <c r="B178" s="31" t="n"/>
-      <c r="C178" s="31" t="n"/>
-      <c r="D178" s="31" t="n"/>
+      <c r="B178" s="34" t="n"/>
+      <c r="C178" s="34" t="n"/>
+      <c r="D178" s="34" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="inlineStr">
@@ -10008,14 +10136,14 @@
       <c r="D184" s="5" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="30" t="inlineStr">
+      <c r="A186" s="33" t="inlineStr">
         <is>
           <t>Heap / Priority Queue</t>
         </is>
       </c>
-      <c r="B186" s="31" t="n"/>
-      <c r="C186" s="31" t="n"/>
-      <c r="D186" s="31" t="n"/>
+      <c r="B186" s="34" t="n"/>
+      <c r="C186" s="34" t="n"/>
+      <c r="D186" s="34" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="inlineStr">
@@ -10124,14 +10252,14 @@
       <c r="D194" s="5" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="30" t="inlineStr">
+      <c r="A196" s="33" t="inlineStr">
         <is>
           <t>Linked List</t>
         </is>
       </c>
-      <c r="B196" s="31" t="n"/>
-      <c r="C196" s="31" t="n"/>
-      <c r="D196" s="31" t="n"/>
+      <c r="B196" s="34" t="n"/>
+      <c r="C196" s="34" t="n"/>
+      <c r="D196" s="34" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="inlineStr">
@@ -10240,14 +10368,14 @@
       <c r="D204" s="5" t="n"/>
     </row>
     <row r="206">
-      <c r="A206" s="30" t="inlineStr">
+      <c r="A206" s="33" t="inlineStr">
         <is>
           <t>Fast &amp; Slow Pointer</t>
         </is>
       </c>
-      <c r="B206" s="31" t="n"/>
-      <c r="C206" s="31" t="n"/>
-      <c r="D206" s="31" t="n"/>
+      <c r="B206" s="34" t="n"/>
+      <c r="C206" s="34" t="n"/>
+      <c r="D206" s="34" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="inlineStr">
@@ -10332,14 +10460,14 @@
       <c r="D212" s="5" t="n"/>
     </row>
     <row r="214">
-      <c r="A214" s="30" t="inlineStr">
+      <c r="A214" s="33" t="inlineStr">
         <is>
           <t>Trees (DFS)</t>
         </is>
       </c>
-      <c r="B214" s="31" t="n"/>
-      <c r="C214" s="31" t="n"/>
-      <c r="D214" s="31" t="n"/>
+      <c r="B214" s="34" t="n"/>
+      <c r="C214" s="34" t="n"/>
+      <c r="D214" s="34" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -10460,14 +10588,14 @@
       <c r="D223" s="7" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="30" t="inlineStr">
+      <c r="A225" s="33" t="inlineStr">
         <is>
           <t>Trees (BFS)</t>
         </is>
       </c>
-      <c r="B225" s="31" t="n"/>
-      <c r="C225" s="31" t="n"/>
-      <c r="D225" s="31" t="n"/>
+      <c r="B225" s="34" t="n"/>
+      <c r="C225" s="34" t="n"/>
+      <c r="D225" s="34" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="inlineStr">
@@ -10564,14 +10692,14 @@
       <c r="D232" s="7" t="n"/>
     </row>
     <row r="234">
-      <c r="A234" s="30" t="inlineStr">
+      <c r="A234" s="33" t="inlineStr">
         <is>
           <t>Binary Search Tree</t>
         </is>
       </c>
-      <c r="B234" s="31" t="n"/>
-      <c r="C234" s="31" t="n"/>
-      <c r="D234" s="31" t="n"/>
+      <c r="B234" s="34" t="n"/>
+      <c r="C234" s="34" t="n"/>
+      <c r="D234" s="34" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
@@ -10668,14 +10796,14 @@
       <c r="D241" s="7" t="n"/>
     </row>
     <row r="243">
-      <c r="A243" s="30" t="inlineStr">
+      <c r="A243" s="33" t="inlineStr">
         <is>
           <t>Graph DFS</t>
         </is>
       </c>
-      <c r="B243" s="31" t="n"/>
-      <c r="C243" s="31" t="n"/>
-      <c r="D243" s="31" t="n"/>
+      <c r="B243" s="34" t="n"/>
+      <c r="C243" s="34" t="n"/>
+      <c r="D243" s="34" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
@@ -10796,14 +10924,14 @@
       <c r="D252" s="7" t="n"/>
     </row>
     <row r="254">
-      <c r="A254" s="30" t="inlineStr">
+      <c r="A254" s="33" t="inlineStr">
         <is>
           <t>Graph BFS</t>
         </is>
       </c>
-      <c r="B254" s="31" t="n"/>
-      <c r="C254" s="31" t="n"/>
-      <c r="D254" s="31" t="n"/>
+      <c r="B254" s="34" t="n"/>
+      <c r="C254" s="34" t="n"/>
+      <c r="D254" s="34" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
@@ -10900,14 +11028,14 @@
       <c r="D261" s="7" t="n"/>
     </row>
     <row r="263">
-      <c r="A263" s="30" t="inlineStr">
+      <c r="A263" s="33" t="inlineStr">
         <is>
           <t>Topological Sort</t>
         </is>
       </c>
-      <c r="B263" s="31" t="n"/>
-      <c r="C263" s="31" t="n"/>
-      <c r="D263" s="31" t="n"/>
+      <c r="B263" s="34" t="n"/>
+      <c r="C263" s="34" t="n"/>
+      <c r="D263" s="34" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
@@ -11004,14 +11132,14 @@
       <c r="D270" s="7" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="30" t="inlineStr">
+      <c r="A272" s="33" t="inlineStr">
         <is>
           <t>Union Find (Disjoint Set)</t>
         </is>
       </c>
-      <c r="B272" s="31" t="n"/>
-      <c r="C272" s="31" t="n"/>
-      <c r="D272" s="31" t="n"/>
+      <c r="B272" s="34" t="n"/>
+      <c r="C272" s="34" t="n"/>
+      <c r="D272" s="34" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
@@ -11120,14 +11248,14 @@
       <c r="D280" s="5" t="n"/>
     </row>
     <row r="282">
-      <c r="A282" s="30" t="inlineStr">
+      <c r="A282" s="33" t="inlineStr">
         <is>
           <t>Trie</t>
         </is>
       </c>
-      <c r="B282" s="31" t="n"/>
-      <c r="C282" s="31" t="n"/>
-      <c r="D282" s="31" t="n"/>
+      <c r="B282" s="34" t="n"/>
+      <c r="C282" s="34" t="n"/>
+      <c r="D282" s="34" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
@@ -11224,14 +11352,14 @@
       <c r="D289" s="7" t="n"/>
     </row>
     <row r="291">
-      <c r="A291" s="30" t="inlineStr">
+      <c r="A291" s="33" t="inlineStr">
         <is>
           <t>Backtracking</t>
         </is>
       </c>
-      <c r="B291" s="31" t="n"/>
-      <c r="C291" s="31" t="n"/>
-      <c r="D291" s="31" t="n"/>
+      <c r="B291" s="34" t="n"/>
+      <c r="C291" s="34" t="n"/>
+      <c r="D291" s="34" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
@@ -11352,14 +11480,14 @@
       <c r="D300" s="7" t="n"/>
     </row>
     <row r="302">
-      <c r="A302" s="30" t="inlineStr">
+      <c r="A302" s="33" t="inlineStr">
         <is>
           <t>Greedy</t>
         </is>
       </c>
-      <c r="B302" s="31" t="n"/>
-      <c r="C302" s="31" t="n"/>
-      <c r="D302" s="31" t="n"/>
+      <c r="B302" s="34" t="n"/>
+      <c r="C302" s="34" t="n"/>
+      <c r="D302" s="34" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
@@ -11468,14 +11596,14 @@
       <c r="D310" s="5" t="n"/>
     </row>
     <row r="312">
-      <c r="A312" s="30" t="inlineStr">
+      <c r="A312" s="33" t="inlineStr">
         <is>
           <t>Dynamic Programming</t>
         </is>
       </c>
-      <c r="B312" s="31" t="n"/>
-      <c r="C312" s="31" t="n"/>
-      <c r="D312" s="31" t="n"/>
+      <c r="B312" s="34" t="n"/>
+      <c r="C312" s="34" t="n"/>
+      <c r="D312" s="34" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
@@ -11608,14 +11736,14 @@
       <c r="D322" s="5" t="n"/>
     </row>
     <row r="324">
-      <c r="A324" s="30" t="inlineStr">
+      <c r="A324" s="33" t="inlineStr">
         <is>
           <t>Interval Problems</t>
         </is>
       </c>
-      <c r="B324" s="31" t="n"/>
-      <c r="C324" s="31" t="n"/>
-      <c r="D324" s="31" t="n"/>
+      <c r="B324" s="34" t="n"/>
+      <c r="C324" s="34" t="n"/>
+      <c r="D324" s="34" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
@@ -11724,14 +11852,14 @@
       <c r="D332" s="5" t="n"/>
     </row>
     <row r="334">
-      <c r="A334" s="30" t="inlineStr">
+      <c r="A334" s="33" t="inlineStr">
         <is>
           <t>Matrix Problems</t>
         </is>
       </c>
-      <c r="B334" s="31" t="n"/>
-      <c r="C334" s="31" t="n"/>
-      <c r="D334" s="31" t="n"/>
+      <c r="B334" s="34" t="n"/>
+      <c r="C334" s="34" t="n"/>
+      <c r="D334" s="34" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
@@ -11828,14 +11956,14 @@
       <c r="D341" s="7" t="n"/>
     </row>
     <row r="343">
-      <c r="A343" s="30" t="inlineStr">
+      <c r="A343" s="33" t="inlineStr">
         <is>
           <t>Design Problems</t>
         </is>
       </c>
-      <c r="B343" s="31" t="n"/>
-      <c r="C343" s="31" t="n"/>
-      <c r="D343" s="31" t="n"/>
+      <c r="B343" s="34" t="n"/>
+      <c r="C343" s="34" t="n"/>
+      <c r="D343" s="34" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="4" t="inlineStr">

</xml_diff>